<commit_message>
renamed EPR and SMR nuclear electricity production datasets
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-nuclear_EPR.xlsx
+++ b/premise/data/additional_inventories/lci-nuclear_EPR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/Github/premise/premise/data/additional_inventories/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/premise/premise/data/additional_inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20D4C7C-9E3D-534A-BF98-C5CF7AF4C6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F15F1E-7A5B-0D4D-A595-19D3023F1417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36540" yWindow="1600" windowWidth="25820" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nuclear electricity" sheetId="1" r:id="rId1"/>
@@ -1334,9 +1334,6 @@
     <t xml:space="preserve">Uranium, enriched 4.8%, at URENCO enrichment plant </t>
   </si>
   <si>
-    <t>electricity production, Evolutionary Power Reactor (EPR)</t>
-  </si>
-  <si>
     <t>1500 MWe, 33.8% electric efficiency. Lifetime of 60 years. Uranium sources: 50% Mng50 % ISL. Uranium enrichment: 4.8%. Fuel burn-up: 60 MWd/kgHM. Simons A, Bauer C. Life cycle assessment of the Evolutionary Power Reactor (EPR) and the influence of different fuel cycle strategies. Proceedings of the Institution of Mechanical Engineers, Part A: Journal of Power and Energy. 2012;226(3):427-444. doi:10.1177/0957650912440549</t>
   </si>
   <si>
@@ -1344,6 +1341,9 @@
   </si>
   <si>
     <t xml:space="preserve">cable, average, EPR </t>
+  </si>
+  <si>
+    <t>electricity production, nuclear, Evolutionary Power Reactor (EPR)</t>
   </si>
 </sst>
 </file>
@@ -1722,7 +1722,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1730,7 +1730,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -2068,7 +2068,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -3468,7 +3468,7 @@
         <v>4</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.2">
@@ -3476,7 +3476,7 @@
         <v>5</v>
       </c>
       <c r="B60" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.2">
@@ -3847,7 +3847,7 @@
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B76">
         <v>1</v>
@@ -5511,7 +5511,7 @@
         <v>4</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="114" spans="1:16" x14ac:dyDescent="0.2">
@@ -5519,7 +5519,7 @@
         <v>5</v>
       </c>
       <c r="B114" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="115" spans="1:16" x14ac:dyDescent="0.2">
@@ -5890,7 +5890,7 @@
     </row>
     <row r="130" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B130">
         <v>1</v>
@@ -7562,7 +7562,7 @@
         <v>5</v>
       </c>
       <c r="B168" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="169" spans="1:16" x14ac:dyDescent="0.2">
@@ -8029,7 +8029,7 @@
         <v>5</v>
       </c>
       <c r="B188" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="189" spans="1:14" x14ac:dyDescent="0.2">
@@ -8496,7 +8496,7 @@
         <v>5</v>
       </c>
       <c r="B208" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="209" spans="1:14" x14ac:dyDescent="0.2">
@@ -8779,7 +8779,7 @@
         <v>5</v>
       </c>
       <c r="B223" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="224" spans="1:14" x14ac:dyDescent="0.2">
@@ -9054,7 +9054,7 @@
         <v>4</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="238" spans="1:14" x14ac:dyDescent="0.2">
@@ -9062,7 +9062,7 @@
         <v>5</v>
       </c>
       <c r="B238" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="239" spans="1:14" x14ac:dyDescent="0.2">
@@ -9086,7 +9086,7 @@
         <v>9</v>
       </c>
       <c r="B241" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="242" spans="1:14" x14ac:dyDescent="0.2">
@@ -9156,7 +9156,7 @@
     </row>
     <row r="246" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B246">
         <v>1</v>
@@ -9180,7 +9180,7 @@
         <v>100</v>
       </c>
       <c r="M246" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="247" spans="1:14" x14ac:dyDescent="0.2">
@@ -9375,7 +9375,7 @@
         <v>4</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="254" spans="1:14" x14ac:dyDescent="0.2">
@@ -9383,7 +9383,7 @@
         <v>5</v>
       </c>
       <c r="B254" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="255" spans="1:14" x14ac:dyDescent="0.2">
@@ -9407,7 +9407,7 @@
         <v>9</v>
       </c>
       <c r="B257" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="258" spans="1:14" x14ac:dyDescent="0.2">
@@ -9477,7 +9477,7 @@
     </row>
     <row r="262" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B262">
         <v>1</v>
@@ -9501,7 +9501,7 @@
         <v>100</v>
       </c>
       <c r="M262" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="263" spans="1:14" x14ac:dyDescent="0.2">
@@ -9704,7 +9704,7 @@
         <v>5</v>
       </c>
       <c r="B270" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="271" spans="1:14" x14ac:dyDescent="0.2">
@@ -10028,7 +10028,7 @@
         <v>5</v>
       </c>
       <c r="B286" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="287" spans="1:14" x14ac:dyDescent="0.2">
@@ -10352,7 +10352,7 @@
         <v>5</v>
       </c>
       <c r="B302" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="303" spans="1:14" x14ac:dyDescent="0.2">
@@ -10638,7 +10638,7 @@
         <v>5</v>
       </c>
       <c r="B317" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="318" spans="1:14" x14ac:dyDescent="0.2">
@@ -11076,7 +11076,7 @@
         <v>5</v>
       </c>
       <c r="B336" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="337" spans="1:14" x14ac:dyDescent="0.2">
@@ -11514,7 +11514,7 @@
         <v>5</v>
       </c>
       <c r="B355" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="356" spans="1:14" x14ac:dyDescent="0.2">
@@ -11838,7 +11838,7 @@
         <v>5</v>
       </c>
       <c r="B371" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="372" spans="1:14" x14ac:dyDescent="0.2">
@@ -12162,7 +12162,7 @@
         <v>5</v>
       </c>
       <c r="B387" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="388" spans="1:14" x14ac:dyDescent="0.2">
@@ -12632,7 +12632,7 @@
         <v>5</v>
       </c>
       <c r="B407" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="408" spans="1:14" x14ac:dyDescent="0.2">
@@ -13102,7 +13102,7 @@
         <v>5</v>
       </c>
       <c r="B427" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="428" spans="1:14" x14ac:dyDescent="0.2">
@@ -13572,7 +13572,7 @@
         <v>5</v>
       </c>
       <c r="B447" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="448" spans="1:14" x14ac:dyDescent="0.2">
@@ -14042,7 +14042,7 @@
         <v>5</v>
       </c>
       <c r="B467" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="468" spans="1:14" x14ac:dyDescent="0.2">
@@ -14794,7 +14794,7 @@
         <v>5</v>
       </c>
       <c r="B499" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="500" spans="1:14" x14ac:dyDescent="0.2">
@@ -15546,7 +15546,7 @@
         <v>5</v>
       </c>
       <c r="B531" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="532" spans="1:14" x14ac:dyDescent="0.2">
@@ -16298,7 +16298,7 @@
         <v>5</v>
       </c>
       <c r="B563" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="564" spans="1:14" x14ac:dyDescent="0.2">
@@ -16619,7 +16619,7 @@
         <v>5</v>
       </c>
       <c r="B579" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="580" spans="1:14" x14ac:dyDescent="0.2">
@@ -16940,7 +16940,7 @@
         <v>5</v>
       </c>
       <c r="B595" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="596" spans="1:14" x14ac:dyDescent="0.2">
@@ -17261,7 +17261,7 @@
         <v>5</v>
       </c>
       <c r="B611" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="612" spans="1:14" x14ac:dyDescent="0.2">
@@ -17547,7 +17547,7 @@
         <v>5</v>
       </c>
       <c r="B626" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="627" spans="1:14" x14ac:dyDescent="0.2">
@@ -17830,7 +17830,7 @@
         <v>5</v>
       </c>
       <c r="B641" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="642" spans="1:14" x14ac:dyDescent="0.2">
@@ -18113,7 +18113,7 @@
         <v>5</v>
       </c>
       <c r="B656" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="657" spans="1:14" x14ac:dyDescent="0.2">
@@ -18332,7 +18332,7 @@
         <v>5</v>
       </c>
       <c r="B669" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="670" spans="1:14" x14ac:dyDescent="0.2">
@@ -18557,7 +18557,7 @@
         <v>5</v>
       </c>
       <c r="B682" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="683" spans="1:15" x14ac:dyDescent="0.2">
@@ -19027,7 +19027,7 @@
         <v>5</v>
       </c>
       <c r="B702" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="703" spans="1:14" x14ac:dyDescent="0.2">
@@ -19497,7 +19497,7 @@
         <v>5</v>
       </c>
       <c r="B722" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="723" spans="1:14" x14ac:dyDescent="0.2">
@@ -19780,7 +19780,7 @@
         <v>5</v>
       </c>
       <c r="B737" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="738" spans="1:14" x14ac:dyDescent="0.2">
@@ -20063,7 +20063,7 @@
         <v>5</v>
       </c>
       <c r="B752" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="753" spans="1:14" x14ac:dyDescent="0.2">
@@ -20419,7 +20419,7 @@
         <v>5</v>
       </c>
       <c r="B769" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="770" spans="1:14" x14ac:dyDescent="0.2">
@@ -20775,7 +20775,7 @@
         <v>5</v>
       </c>
       <c r="B786" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="787" spans="1:14" x14ac:dyDescent="0.2">
@@ -21131,7 +21131,7 @@
         <v>5</v>
       </c>
       <c r="B803" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="804" spans="1:14" x14ac:dyDescent="0.2">
@@ -21487,7 +21487,7 @@
         <v>5</v>
       </c>
       <c r="B820" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="821" spans="1:14" x14ac:dyDescent="0.2">
@@ -21843,7 +21843,7 @@
         <v>5</v>
       </c>
       <c r="B837" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="838" spans="1:14" x14ac:dyDescent="0.2">
@@ -22199,7 +22199,7 @@
         <v>5</v>
       </c>
       <c r="B854" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="855" spans="1:14" x14ac:dyDescent="0.2">
@@ -22935,7 +22935,7 @@
         <v>5</v>
       </c>
       <c r="B881" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="882" spans="1:14" x14ac:dyDescent="0.2">
@@ -23671,7 +23671,7 @@
         <v>5</v>
       </c>
       <c r="B908" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="909" spans="1:14" x14ac:dyDescent="0.2">
@@ -23954,7 +23954,7 @@
         <v>5</v>
       </c>
       <c r="B923" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="924" spans="1:14" x14ac:dyDescent="0.2">
@@ -24237,7 +24237,7 @@
         <v>5</v>
       </c>
       <c r="B938" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="939" spans="1:14" x14ac:dyDescent="0.2">
@@ -24523,7 +24523,7 @@
         <v>5</v>
       </c>
       <c r="B953" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="954" spans="1:16" x14ac:dyDescent="0.2">
@@ -26093,7 +26093,7 @@
         <v>5</v>
       </c>
       <c r="B1001" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1002" spans="1:16" x14ac:dyDescent="0.2">
@@ -27663,7 +27663,7 @@
         <v>5</v>
       </c>
       <c r="B1049" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1050" spans="1:16" x14ac:dyDescent="0.2">
@@ -27987,7 +27987,7 @@
         <v>5</v>
       </c>
       <c r="B1065" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1066" spans="1:14" x14ac:dyDescent="0.2">
@@ -28311,7 +28311,7 @@
         <v>5</v>
       </c>
       <c r="B1081" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1082" spans="1:14" x14ac:dyDescent="0.2">
@@ -28434,7 +28434,7 @@
     </row>
     <row r="1090" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1090" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B1090">
         <v>262500</v>
@@ -28461,7 +28461,7 @@
         <v>262500</v>
       </c>
       <c r="M1090" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="1091" spans="1:13" x14ac:dyDescent="0.2">
@@ -29281,7 +29281,7 @@
         <v>5</v>
       </c>
       <c r="B1117" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1118" spans="1:14" x14ac:dyDescent="0.2">
@@ -29404,7 +29404,7 @@
     </row>
     <row r="1126" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1126" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B1126">
         <v>262500</v>
@@ -29431,7 +29431,7 @@
         <v>262500</v>
       </c>
       <c r="M1126" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="1127" spans="1:14" x14ac:dyDescent="0.2">
@@ -30175,7 +30175,7 @@
         <v>5</v>
       </c>
       <c r="B1151" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1152" spans="1:14" x14ac:dyDescent="0.2">
@@ -30499,7 +30499,7 @@
         <v>5</v>
       </c>
       <c r="B1167" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1168" spans="1:14" x14ac:dyDescent="0.2">
@@ -30823,7 +30823,7 @@
         <v>5</v>
       </c>
       <c r="B1183" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1184" spans="1:14" x14ac:dyDescent="0.2">
@@ -31182,7 +31182,7 @@
         <v>5</v>
       </c>
       <c r="B1200" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1201" spans="1:14" x14ac:dyDescent="0.2">
@@ -31468,7 +31468,7 @@
         <v>5</v>
       </c>
       <c r="B1215" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1216" spans="1:14" x14ac:dyDescent="0.2">
@@ -31754,7 +31754,7 @@
         <v>5</v>
       </c>
       <c r="B1230" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1231" spans="1:14" x14ac:dyDescent="0.2">
@@ -32078,7 +32078,7 @@
         <v>5</v>
       </c>
       <c r="B1246" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1247" spans="1:14" x14ac:dyDescent="0.2">
@@ -32478,7 +32478,7 @@
         <v>5</v>
       </c>
       <c r="B1264" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1265" spans="1:14" x14ac:dyDescent="0.2">
@@ -32764,7 +32764,7 @@
         <v>5</v>
       </c>
       <c r="B1279" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1280" spans="1:14" x14ac:dyDescent="0.2">
@@ -33052,7 +33052,7 @@
         <v>5</v>
       </c>
       <c r="B1295" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1296" spans="1:12" x14ac:dyDescent="0.2">
@@ -33308,7 +33308,7 @@
         <v>5</v>
       </c>
       <c r="B1310" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1311" spans="1:12" x14ac:dyDescent="0.2">
@@ -33564,7 +33564,7 @@
         <v>5</v>
       </c>
       <c r="B1325" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1326" spans="1:12" x14ac:dyDescent="0.2">
@@ -34002,7 +34002,7 @@
         <v>5</v>
       </c>
       <c r="B1344" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1345" spans="1:14" x14ac:dyDescent="0.2">
@@ -34402,7 +34402,7 @@
         <v>5</v>
       </c>
       <c r="B1362" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1363" spans="1:14" x14ac:dyDescent="0.2">
@@ -34589,7 +34589,7 @@
     </row>
     <row r="1373" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1373" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B1373">
         <v>150000</v>
@@ -34616,7 +34616,7 @@
         <v>150000</v>
       </c>
       <c r="M1373" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="1374" spans="1:14" x14ac:dyDescent="0.2">
@@ -35022,7 +35022,7 @@
         <v>5</v>
       </c>
       <c r="B1388" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1389" spans="1:14" x14ac:dyDescent="0.2">
@@ -35209,7 +35209,7 @@
     </row>
     <row r="1399" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1399" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B1399">
         <v>150000</v>
@@ -35236,7 +35236,7 @@
         <v>150000</v>
       </c>
       <c r="M1399" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="1400" spans="1:14" x14ac:dyDescent="0.2">
@@ -35642,7 +35642,7 @@
         <v>5</v>
       </c>
       <c r="B1414" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1415" spans="1:14" x14ac:dyDescent="0.2">
@@ -36076,7 +36076,7 @@
         <v>5</v>
       </c>
       <c r="B1434" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1435" spans="1:14" x14ac:dyDescent="0.2">
@@ -36472,7 +36472,7 @@
         <v>5</v>
       </c>
       <c r="B1453" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1454" spans="1:14" x14ac:dyDescent="0.2">
@@ -36980,7 +36980,7 @@
         <v>5</v>
       </c>
       <c r="B1474" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1475" spans="1:14" x14ac:dyDescent="0.2">
@@ -37450,7 +37450,7 @@
         <v>5</v>
       </c>
       <c r="B1494" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1495" spans="1:14" x14ac:dyDescent="0.2">
@@ -37809,7 +37809,7 @@
         <v>5</v>
       </c>
       <c r="B1511" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1512" spans="1:14" x14ac:dyDescent="0.2">
@@ -38133,7 +38133,7 @@
         <v>5</v>
       </c>
       <c r="B1527" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1528" spans="1:14" x14ac:dyDescent="0.2">
@@ -38419,7 +38419,7 @@
         <v>5</v>
       </c>
       <c r="B1542" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1543" spans="1:14" x14ac:dyDescent="0.2">
@@ -38705,7 +38705,7 @@
         <v>5</v>
       </c>
       <c r="B1557" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1558" spans="1:14" x14ac:dyDescent="0.2">
@@ -39502,7 +39502,7 @@
         <v>5</v>
       </c>
       <c r="B1586" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1587" spans="1:14" x14ac:dyDescent="0.2">
@@ -40299,7 +40299,7 @@
         <v>5</v>
       </c>
       <c r="B1615" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1616" spans="1:14" x14ac:dyDescent="0.2">
@@ -40807,7 +40807,7 @@
         <v>5</v>
       </c>
       <c r="B1636" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1637" spans="1:14" x14ac:dyDescent="0.2">
@@ -41315,7 +41315,7 @@
         <v>5</v>
       </c>
       <c r="B1657" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1658" spans="1:14" x14ac:dyDescent="0.2">
@@ -42051,7 +42051,7 @@
         <v>5</v>
       </c>
       <c r="B1684" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1685" spans="1:14" x14ac:dyDescent="0.2">
@@ -42787,7 +42787,7 @@
         <v>5</v>
       </c>
       <c r="B1711" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1712" spans="1:14" x14ac:dyDescent="0.2">
@@ -43146,7 +43146,7 @@
         <v>5</v>
       </c>
       <c r="B1728" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1729" spans="1:14" x14ac:dyDescent="0.2">
@@ -43692,7 +43692,7 @@
         <v>5</v>
       </c>
       <c r="B1750" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1751" spans="1:14" x14ac:dyDescent="0.2">
@@ -44238,7 +44238,7 @@
         <v>5</v>
       </c>
       <c r="B1772" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1773" spans="1:14" x14ac:dyDescent="0.2">
@@ -44974,7 +44974,7 @@
         <v>5</v>
       </c>
       <c r="B1799" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1800" spans="1:14" x14ac:dyDescent="0.2">
@@ -45710,7 +45710,7 @@
         <v>5</v>
       </c>
       <c r="B1826" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1827" spans="1:14" x14ac:dyDescent="0.2">
@@ -45996,7 +45996,7 @@
         <v>5</v>
       </c>
       <c r="B1841" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1842" spans="1:14" x14ac:dyDescent="0.2">
@@ -46282,7 +46282,7 @@
         <v>5</v>
       </c>
       <c r="B1856" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1857" spans="1:14" x14ac:dyDescent="0.2">
@@ -47716,7 +47716,7 @@
         <v>5</v>
       </c>
       <c r="B1905" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1906" spans="1:14" x14ac:dyDescent="0.2">
@@ -49150,7 +49150,7 @@
         <v>5</v>
       </c>
       <c r="B1954" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="1955" spans="1:14" x14ac:dyDescent="0.2">
@@ -51021,7 +51021,7 @@
         <v>5</v>
       </c>
       <c r="B2013" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="2014" spans="1:14" x14ac:dyDescent="0.2">
@@ -52892,7 +52892,7 @@
         <v>5</v>
       </c>
       <c r="B2072" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="2073" spans="1:14" x14ac:dyDescent="0.2">
@@ -53251,7 +53251,7 @@
         <v>5</v>
       </c>
       <c r="B2089" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="2090" spans="1:14" x14ac:dyDescent="0.2">
@@ -53727,7 +53727,7 @@
         <v>5</v>
       </c>
       <c r="B2109" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="2110" spans="1:14" x14ac:dyDescent="0.2">

</xml_diff>